<commit_message>
Fix department dropdowns to load from departmentlocks instead of activities
</commit_message>
<xml_diff>
--- a/ฐานข้อมูลกิจกรรม.xlsx
+++ b/ฐานข้อมูลกิจกรรม.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3ad82ec08daddac8/Documents/Budget70/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="69" documentId="8_{508F8A76-7266-4C03-96A4-7FC4074F897A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0DB4EA59-D933-4472-BC81-3DDC15904F7C}"/>
+  <xr:revisionPtr revIDLastSave="105" documentId="8_{508F8A76-7266-4C03-96A4-7FC4074F897A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{438787AF-27B7-470E-8B5F-F861CED3EE30}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{03DD3A07-A8AA-43B7-820F-79B2DA53CF56}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="108">
   <si>
     <t>activity_id</t>
   </si>
@@ -62,72 +62,6 @@
     <t>บว01</t>
   </si>
   <si>
-    <t>บริหารวิชาการ</t>
-  </si>
-  <si>
-    <t>บริหารงบประมาณและแผนงาน(งานการเงิน)</t>
-  </si>
-  <si>
-    <t>บริหารงบประมาณและแผนงาน(งานแผนงาน)</t>
-  </si>
-  <si>
-    <t>บริหารงบประมาณและแผนงาน(งานพัสดุ)</t>
-  </si>
-  <si>
-    <t>บริหารงบประมาณและแผนงาน(งานยานพาหนะ)</t>
-  </si>
-  <si>
-    <t>บริหารงบประมาณและแผนงาน(งานโรงเรียนธนาคาร)</t>
-  </si>
-  <si>
-    <t>บริหารทั่วไป</t>
-  </si>
-  <si>
-    <t>บริหารอำนวยการและบุคคล</t>
-  </si>
-  <si>
-    <t>ภาษาไทย</t>
-  </si>
-  <si>
-    <t>คณิตศาสตร์</t>
-  </si>
-  <si>
-    <t>วิทยาศาสตร์</t>
-  </si>
-  <si>
-    <t>เทคโนโลยี</t>
-  </si>
-  <si>
-    <t>สังคมศึกษา</t>
-  </si>
-  <si>
-    <t>การงานอาชีพ</t>
-  </si>
-  <si>
-    <t>สุขศึกษา</t>
-  </si>
-  <si>
-    <t>ภาษาต่างประเทศ</t>
-  </si>
-  <si>
-    <t>กิจกรรมพัฒนาผู้เรียน</t>
-  </si>
-  <si>
-    <t>แนะแนว</t>
-  </si>
-  <si>
-    <t>ห้องสมุด</t>
-  </si>
-  <si>
-    <t>บริหารกิจการนักเรียน</t>
-  </si>
-  <si>
-    <t>ห้องเรียนพิเศษ</t>
-  </si>
-  <si>
-    <t>ศิลปะ</t>
-  </si>
-  <si>
     <t>บง01</t>
   </si>
   <si>
@@ -140,9 +74,6 @@
     <t>บง04</t>
   </si>
   <si>
-    <t>บง05</t>
-  </si>
-  <si>
     <t>บท01</t>
   </si>
   <si>
@@ -327,6 +258,111 @@
   </si>
   <si>
     <t>บุคคล22</t>
+  </si>
+  <si>
+    <t>1.กลุ่มบริหารวิชาการ</t>
+  </si>
+  <si>
+    <t>2.1 กลุ่มบริหารงบประมาณและแผนงาน (งานการเงินและบัญชี)</t>
+  </si>
+  <si>
+    <t>2.2 กลุ่มบริหารงบประมาณและแผนงาน (งานแผนงาน)</t>
+  </si>
+  <si>
+    <t>2.3 กลุ่มบริหารงบประมาณและแผนงาน (งานพัสดุ)</t>
+  </si>
+  <si>
+    <t>2.4 กลุ่มบริหารงบประมาณและแผนงาน (งานโรงเรียนธนาคาร)</t>
+  </si>
+  <si>
+    <t>3.1 กลุ่มบริหารอำนวยการและบุคคล (งานสารบรรณ)</t>
+  </si>
+  <si>
+    <t>3.2 กลุ่มบริหารอำนวยการและบุคคล (งานบุคคล)</t>
+  </si>
+  <si>
+    <t>3.3 กลุ่มบริหารอำนวยการและบุคคล (งานควบคุมภายใน)</t>
+  </si>
+  <si>
+    <t>4.1 กลุ่มบริหารทั่วไป (สำนักงาน)</t>
+  </si>
+  <si>
+    <t>4.2  กลุ่มบริหารทั่วไป (งานโสตทัศนูปกรณ์)</t>
+  </si>
+  <si>
+    <t>5.1 กลุ่มบริหารกิจการนักเรียน (สำนักงาน)</t>
+  </si>
+  <si>
+    <t>5.2 กลุ่มบริหารกิจการนักเรียน (สภานักเรียน)</t>
+  </si>
+  <si>
+    <t>6. โครงการห้องเรียนวิทยาศาสตร์พลังสิบ</t>
+  </si>
+  <si>
+    <t>7. กลุ่มสาระการเรียนรู้ภาษาไทย</t>
+  </si>
+  <si>
+    <t>8. กลุ่มสาระการเรียนรู้คณิตศาสตร์</t>
+  </si>
+  <si>
+    <t>9.กลุ่มสาระการเรียนรู้วิทยาศาสตร์และเทคโนโลยี</t>
+  </si>
+  <si>
+    <t>10.งานคอมพิวเตอร์</t>
+  </si>
+  <si>
+    <t>11.กลุ่มสาระการเรียนรู้สังคมศึกษา ศาสนาและวัฒนธรรม</t>
+  </si>
+  <si>
+    <t>12.กลุ่มสาระการเรียนรู้สุขศึกษาและพลศึกษา</t>
+  </si>
+  <si>
+    <t>13.กลุ่มสาระการเรียนรู้ศิลปะ</t>
+  </si>
+  <si>
+    <t>14.กลุ่มสาระการเรียนรู้ภาษาต่างประเทศ</t>
+  </si>
+  <si>
+    <t>15.กลุ่มสาระการเรียนรู้การงานอาชีพ</t>
+  </si>
+  <si>
+    <t>16.งานกิจกรรมพัฒนาผู้เรียน</t>
+  </si>
+  <si>
+    <t>17.งานแนะแนว</t>
+  </si>
+  <si>
+    <t>18.งานห้องสมุด</t>
+  </si>
+  <si>
+    <t>ทดลองระบบ23</t>
+  </si>
+  <si>
+    <t>ทดลองระบบ24</t>
+  </si>
+  <si>
+    <t>ทดลองระบบ25</t>
+  </si>
+  <si>
+    <t>บุคคล23</t>
+  </si>
+  <si>
+    <t>บุคคล24</t>
+  </si>
+  <si>
+    <t>บุคคล25</t>
+  </si>
+  <si>
+    <t>บค02</t>
+  </si>
+  <si>
+    <t>บท02</t>
+  </si>
+  <si>
+    <t>ขค03</t>
+  </si>
+  <si>
+    <t>บก02</t>
   </si>
 </sst>
 </file>
@@ -401,6 +437,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -720,7 +760,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80C65560-D526-4562-81E7-DD6D72ECE788}">
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.5" bestFit="1" customWidth="1"/>
@@ -755,439 +795,499 @@
         <v>6</v>
       </c>
       <c r="B2" t="s">
-        <v>50</v>
+        <v>27</v>
       </c>
       <c r="C2" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D2" t="s">
+        <v>29</v>
+      </c>
+      <c r="E2" t="s">
+        <v>73</v>
+      </c>
+      <c r="F2" t="s">
         <v>51</v>
-      </c>
-      <c r="D2" t="s">
-        <v>52</v>
-      </c>
-      <c r="E2" t="s">
-        <v>7</v>
-      </c>
-      <c r="F2" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>29</v>
+        <v>7</v>
       </c>
       <c r="B3" t="s">
-        <v>50</v>
+        <v>27</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>51</v>
+        <v>28</v>
       </c>
       <c r="D3" t="s">
-        <v>53</v>
+        <v>30</v>
       </c>
       <c r="E3" t="s">
-        <v>8</v>
+        <v>74</v>
       </c>
       <c r="F3" t="s">
-        <v>75</v>
+        <v>52</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="B4" t="s">
-        <v>50</v>
+        <v>27</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>51</v>
+        <v>28</v>
       </c>
       <c r="D4" t="s">
-        <v>54</v>
+        <v>31</v>
       </c>
       <c r="E4" t="s">
-        <v>9</v>
+        <v>75</v>
       </c>
       <c r="F4" t="s">
-        <v>76</v>
+        <v>53</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>31</v>
+        <v>9</v>
       </c>
       <c r="B5" t="s">
-        <v>50</v>
+        <v>27</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>51</v>
+        <v>28</v>
       </c>
       <c r="D5" t="s">
-        <v>55</v>
+        <v>32</v>
       </c>
       <c r="E5" t="s">
-        <v>10</v>
+        <v>76</v>
       </c>
       <c r="F5" t="s">
-        <v>77</v>
+        <v>54</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>32</v>
+        <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>50</v>
+        <v>27</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>51</v>
+        <v>28</v>
       </c>
       <c r="D6" t="s">
-        <v>56</v>
+        <v>33</v>
       </c>
       <c r="E6" t="s">
-        <v>11</v>
+        <v>77</v>
       </c>
       <c r="F6" t="s">
-        <v>78</v>
+        <v>55</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>33</v>
+        <v>12</v>
       </c>
       <c r="B7" t="s">
-        <v>50</v>
+        <v>27</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>51</v>
+        <v>28</v>
       </c>
       <c r="D7" t="s">
-        <v>57</v>
+        <v>34</v>
       </c>
       <c r="E7" t="s">
-        <v>12</v>
+        <v>78</v>
       </c>
       <c r="F7" t="s">
-        <v>79</v>
+        <v>56</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>34</v>
+        <v>104</v>
       </c>
       <c r="B8" t="s">
-        <v>50</v>
+        <v>27</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>51</v>
+        <v>28</v>
       </c>
       <c r="D8" t="s">
-        <v>58</v>
+        <v>35</v>
       </c>
       <c r="E8" t="s">
-        <v>13</v>
+        <v>79</v>
       </c>
       <c r="F8" t="s">
-        <v>80</v>
+        <v>57</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
+        <v>106</v>
+      </c>
+      <c r="B9" t="s">
+        <v>27</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D9" t="s">
         <v>36</v>
       </c>
-      <c r="B9" t="s">
-        <v>50</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="D9" t="s">
-        <v>59</v>
-      </c>
       <c r="E9" t="s">
-        <v>26</v>
+        <v>80</v>
       </c>
       <c r="F9" t="s">
-        <v>81</v>
+        <v>58</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>35</v>
+        <v>11</v>
       </c>
       <c r="B10" t="s">
-        <v>50</v>
+        <v>27</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>51</v>
+        <v>28</v>
       </c>
       <c r="D10" t="s">
-        <v>60</v>
+        <v>37</v>
       </c>
       <c r="E10" t="s">
-        <v>14</v>
+        <v>81</v>
       </c>
       <c r="F10" t="s">
-        <v>82</v>
+        <v>59</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>37</v>
+        <v>105</v>
       </c>
       <c r="B11" t="s">
-        <v>50</v>
+        <v>27</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>51</v>
+        <v>28</v>
       </c>
       <c r="D11" t="s">
-        <v>61</v>
+        <v>38</v>
       </c>
       <c r="E11" t="s">
-        <v>15</v>
+        <v>82</v>
       </c>
       <c r="F11" t="s">
-        <v>83</v>
+        <v>60</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>38</v>
+        <v>13</v>
       </c>
       <c r="B12" t="s">
-        <v>50</v>
+        <v>27</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>51</v>
+        <v>28</v>
       </c>
       <c r="D12" t="s">
-        <v>62</v>
+        <v>39</v>
       </c>
       <c r="E12" t="s">
-        <v>16</v>
+        <v>83</v>
       </c>
       <c r="F12" t="s">
-        <v>84</v>
+        <v>61</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>39</v>
+        <v>107</v>
       </c>
       <c r="B13" t="s">
-        <v>50</v>
+        <v>27</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>51</v>
+        <v>28</v>
       </c>
       <c r="D13" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="E13" t="s">
-        <v>17</v>
+        <v>84</v>
       </c>
       <c r="F13" t="s">
-        <v>85</v>
+        <v>62</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="B14" t="s">
-        <v>50</v>
+        <v>27</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>51</v>
+        <v>28</v>
       </c>
       <c r="D14" t="s">
-        <v>64</v>
+        <v>41</v>
       </c>
       <c r="E14" t="s">
-        <v>18</v>
+        <v>85</v>
       </c>
       <c r="F14" t="s">
-        <v>86</v>
+        <v>63</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>41</v>
+        <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>50</v>
+        <v>27</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>51</v>
+        <v>28</v>
       </c>
       <c r="D15" t="s">
-        <v>65</v>
+        <v>42</v>
       </c>
       <c r="E15" t="s">
-        <v>19</v>
+        <v>86</v>
       </c>
       <c r="F15" t="s">
-        <v>87</v>
+        <v>64</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>42</v>
+        <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>50</v>
+        <v>27</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>51</v>
+        <v>28</v>
       </c>
       <c r="D16" t="s">
-        <v>66</v>
+        <v>43</v>
       </c>
       <c r="E16" t="s">
-        <v>20</v>
+        <v>87</v>
       </c>
       <c r="F16" t="s">
-        <v>88</v>
+        <v>65</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>43</v>
+        <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>50</v>
+        <v>27</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>51</v>
+        <v>28</v>
       </c>
       <c r="D17" t="s">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="E17" t="s">
-        <v>21</v>
+        <v>88</v>
       </c>
       <c r="F17" t="s">
-        <v>89</v>
+        <v>66</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>44</v>
+        <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>50</v>
+        <v>27</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>51</v>
+        <v>28</v>
       </c>
       <c r="D18" t="s">
-        <v>68</v>
+        <v>45</v>
       </c>
       <c r="E18" t="s">
-        <v>22</v>
+        <v>89</v>
       </c>
       <c r="F18" t="s">
-        <v>90</v>
+        <v>67</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>45</v>
+        <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>50</v>
+        <v>27</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>51</v>
+        <v>28</v>
       </c>
       <c r="D19" t="s">
-        <v>69</v>
+        <v>46</v>
       </c>
       <c r="E19" t="s">
-        <v>24</v>
+        <v>90</v>
       </c>
       <c r="F19" t="s">
-        <v>91</v>
+        <v>68</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>46</v>
+        <v>20</v>
       </c>
       <c r="B20" t="s">
-        <v>50</v>
+        <v>27</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>51</v>
+        <v>28</v>
       </c>
       <c r="D20" t="s">
-        <v>70</v>
+        <v>47</v>
       </c>
       <c r="E20" t="s">
-        <v>25</v>
+        <v>91</v>
       </c>
       <c r="F20" t="s">
-        <v>92</v>
+        <v>69</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>47</v>
+        <v>26</v>
       </c>
       <c r="B21" t="s">
-        <v>50</v>
+        <v>27</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>51</v>
+        <v>28</v>
       </c>
       <c r="D21" t="s">
-        <v>71</v>
+        <v>48</v>
       </c>
       <c r="E21" t="s">
-        <v>23</v>
+        <v>92</v>
       </c>
       <c r="F21" t="s">
-        <v>93</v>
+        <v>70</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>48</v>
+        <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>50</v>
+        <v>27</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>51</v>
+        <v>28</v>
       </c>
       <c r="D22" t="s">
-        <v>72</v>
+        <v>49</v>
       </c>
       <c r="E22" t="s">
-        <v>27</v>
+        <v>93</v>
       </c>
       <c r="F22" t="s">
-        <v>94</v>
+        <v>71</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>49</v>
+        <v>19</v>
       </c>
       <c r="B23" t="s">
+        <v>27</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D23" t="s">
         <v>50</v>
       </c>
-      <c r="C23" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="D23" t="s">
-        <v>73</v>
-      </c>
       <c r="E23" t="s">
-        <v>28</v>
+        <v>94</v>
       </c>
       <c r="F23" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>24</v>
+      </c>
+      <c r="B24" t="s">
+        <v>27</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D24" t="s">
+        <v>98</v>
+      </c>
+      <c r="E24" t="s">
         <v>95</v>
+      </c>
+      <c r="F24" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>22</v>
+      </c>
+      <c r="B25" t="s">
+        <v>27</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D25" t="s">
+        <v>99</v>
+      </c>
+      <c r="E25" t="s">
+        <v>96</v>
+      </c>
+      <c r="F25" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>23</v>
+      </c>
+      <c r="B26" t="s">
+        <v>27</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D26" t="s">
+        <v>100</v>
+      </c>
+      <c r="E26" t="s">
+        <v>97</v>
+      </c>
+      <c r="F26" t="s">
+        <v>103</v>
       </c>
     </row>
   </sheetData>

</xml_diff>